<commit_message>
feat: halve welding points below 8 booths
</commit_message>
<xml_diff>
--- a/data/xlsx/aeosib--welding-and-fabrication-1g-2g-and-3g.xlsx
+++ b/data/xlsx/aeosib--welding-and-fabrication-1g-2g-and-3g.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -58,6 +58,10 @@
       <name val="Arial"/>
       <charset val="1"/>
       <family val="0"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -136,7 +140,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -226,6 +230,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -480,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15.17" customWidth="1" style="15" min="1" max="1"/>
@@ -1056,9 +1063,17 @@
         </is>
       </c>
     </row>
+    <row r="36" ht="14.15" customHeight="1" s="16">
+      <c r="A36" s="32" t="inlineStr">
+        <is>
+          <t>* For this course, the institute should have at least 8 welding booths. Otherwise, the total points achieved will be halved.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A36:G36"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A1:G1"/>

</xml_diff>